<commit_message>
Evento #3 registrado en reporte_2026-06-14.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-14.xlsx
+++ b/datos/excel/reporte_2026-06-14.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,6 +513,51 @@
         <v>6126</v>
       </c>
       <c r="K2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>12:26:33</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>144</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>312.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-15.78</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>578.1 Hz | 898.4 Hz | 1210.9 Hz</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>2527</v>
+      </c>
+      <c r="J3" t="n">
+        <v>60</v>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Evento #4 registrado en reporte_2026-06-14.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-14.xlsx
+++ b/datos/excel/reporte_2026-06-14.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,51 @@
         <v>60</v>
       </c>
       <c r="K3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>12:26:42</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>304.69</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-10.44</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>578.1 Hz | 945.3 Hz | 1187.5 Hz</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>2510</v>
+      </c>
+      <c r="J4" t="n">
+        <v>60</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Evento #5 registrado en reporte_2026-06-14.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-14.xlsx
+++ b/datos/excel/reporte_2026-06-14.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -603,6 +603,51 @@
         <v>60</v>
       </c>
       <c r="K4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>12:26:51</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>312.5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-16.38</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>585.9 Hz | 953.1 Hz | 1210.9 Hz</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>2514</v>
+      </c>
+      <c r="J5" t="n">
+        <v>62</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Evento #6 registrado en reporte_2026-06-14.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-14.xlsx
+++ b/datos/excel/reporte_2026-06-14.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,6 +648,51 @@
         <v>62</v>
       </c>
       <c r="K5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>12:26:58</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>320.31</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-16.15</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>609.4 Hz | 1007.8 Hz | 1265.6 Hz</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>2529</v>
+      </c>
+      <c r="J6" t="n">
+        <v>60</v>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Evento #7 registrado en reporte_2026-06-14.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-14.xlsx
+++ b/datos/excel/reporte_2026-06-14.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -693,6 +693,51 @@
         <v>60</v>
       </c>
       <c r="K6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>12:27:09</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>147</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>335.94</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-17.36</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>718.8 Hz | 1039.1 Hz | 1382.8 Hz</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>2536</v>
+      </c>
+      <c r="J7" t="n">
+        <v>62</v>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Evento #8 registrado en reporte_2026-06-14.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-14.xlsx
+++ b/datos/excel/reporte_2026-06-14.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -738,6 +738,51 @@
         <v>62</v>
       </c>
       <c r="K7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>12:27:22</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>144</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>273.44</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-18.05</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>515.6 Hz | 773.4 Hz | 1054.7 Hz</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>2548</v>
+      </c>
+      <c r="J8" t="n">
+        <v>60</v>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Evento #9 registrado en reporte_2026-06-14.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-14.xlsx
+++ b/datos/excel/reporte_2026-06-14.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -783,6 +783,51 @@
         <v>60</v>
       </c>
       <c r="K8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>12:27:37</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>320.31</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-12.45</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>687.5 Hz | 1000.0 Hz | 1296.9 Hz</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>2899</v>
+      </c>
+      <c r="J9" t="n">
+        <v>60</v>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Evento #10 registrado en reporte_2026-06-14.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-14.xlsx
+++ b/datos/excel/reporte_2026-06-14.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -833,6 +833,51 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>12:27:46</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>312.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-16.19</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>601.6 Hz | 968.8 Hz | 1203.1 Hz</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>2562</v>
+      </c>
+      <c r="J10" t="n">
+        <v>59</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Evento #11 registrado en reporte_2026-06-14.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-14.xlsx
+++ b/datos/excel/reporte_2026-06-14.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -878,6 +878,51 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>11</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>12:27:53</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>328.12</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-15.57</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>609.4 Hz | 1031.2 Hz | 1265.6 Hz</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>2539</v>
+      </c>
+      <c r="J11" t="n">
+        <v>61</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Evento #12 registrado en reporte_2026-06-14.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-14.xlsx
+++ b/datos/excel/reporte_2026-06-14.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -923,6 +923,51 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>12</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>12:28:01</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>138</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>335.94</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-17.07</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>718.8 Hz | 1031.2 Hz | 1390.6 Hz</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>2555</v>
+      </c>
+      <c r="J12" t="n">
+        <v>59</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Evento #13 registrado en reporte_2026-06-14.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-14.xlsx
+++ b/datos/excel/reporte_2026-06-14.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -968,6 +968,51 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>13</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>12:28:37</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>281.25</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-16.36</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>515.6 Hz | 796.9 Hz | 1078.1 Hz</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>2560</v>
+      </c>
+      <c r="J13" t="n">
+        <v>60</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Evento #1 registrado en reporte_2026-06-14.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-14.xlsx
+++ b/datos/excel/reporte_2026-06-14.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1013,6 +1013,51 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>12:30:35</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>320.31</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-9.039999999999999</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>609.4 Hz | 992.2 Hz | 1234.4 Hz</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>2520</v>
+      </c>
+      <c r="J14" t="n">
+        <v>11133</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>